<commit_message>
feat(schema): render VoID with its own names and IRIs, in this project's words
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/void.xlsx
+++ b/project/excel/void.xlsx
@@ -7,12 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="resource" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="dataset" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="document" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="dataset description" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="linkset" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="technical feature" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Dataset" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Linkset" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="DatasetDescription" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="TechnicalFeature" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ClassBasedPartition" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="PropertyBasedPartition" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,9 +418,182 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:AH1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>creator</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>contributor</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>publisher</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>created</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>issued</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>license</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>subject</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>homepage</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>feature</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>sparqlEndpoint</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>dataDump</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>uriLookupEndpoint</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>openSearchDescription</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>rootResource</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>exampleResource</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>uriSpace</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>uriRegexPattern</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>vocabulary</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>subset</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>classPartition</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>propertyPartition</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>triples</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>entities</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>classes</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>properties</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>distinctSubjects</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>distinctObjects</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -431,9 +604,202 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:AL1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>subjectsTarget</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>objectsTarget</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>linkPredicate</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>creator</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>contributor</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>publisher</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>created</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>issued</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>license</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>subject</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>homepage</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>feature</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>sparqlEndpoint</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>dataDump</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>uriLookupEndpoint</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>openSearchDescription</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>rootResource</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>exampleResource</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>uriSpace</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>uriRegexPattern</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>vocabulary</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>subset</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>classPartition</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>propertyPartition</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>triples</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>entities</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>classes</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>properties</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>distinctSubjects</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>distinctObjects</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -444,9 +810,57 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>creator</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>created</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>primaryTopic</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>inDataset</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -457,9 +871,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>seeAlso</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -470,9 +907,57 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>triples</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>entities</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>classes</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>properties</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>distinctSubjects</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>distinctObjects</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>propertyPartition</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -483,9 +968,52 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>property</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>triples</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>entities</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>classes</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>properties</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>distinctSubjects</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>distinctObjects</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>